<commit_message>
feat: add multiple delivery destinations
</commit_message>
<xml_diff>
--- a/project_clinic_order_management_db_definition.xlsx
+++ b/project_clinic_order_management_db_definition.xlsx
@@ -290,7 +290,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Supabaseのpatient_orders / patient_order_items / order_shipping_addresses / patient_order_events</t>
+          <t xml:space="preserve">Supabaseのpatient_orders / patient_order_items / delivery_destinations / order_delivery_destinations / patient_order_events</t>
         </is>
       </c>
     </row>
@@ -338,7 +338,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">自宅配送時はorder_shipping_addressesへ注文時点の配送先を保存し、住所なし配送を拒否する。</t>
+          <t xml:space="preserve">医院・患者は複数送り先を持ち、order_delivery_destinationsへ注文時点の送り先を保存する。</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -701,12 +701,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">自宅配送注文に対して、注文時点の配送先を1対1で保存する履歴スナップショット。</t>
+          <t xml:space="preserve">医院または患者が複数所有できる送り先。論理削除と既定送り先を管理する。</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">order_delivery_destinations</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文登録と状態変更について、操作者と変更前後の状態を保存する監査イベント。</t>
+          <t xml:space="preserve">選択した送り先を注文時点の不変スナップショットとして1対1で保存する。</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -760,27 +760,27 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">patient_order_events</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
+          <t xml:space="preserve">注文登録と状態変更について、操作者と変更前後の状態を保存する監査イベント。</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文拡張</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存テーブル拡張案</t>
+          <t xml:space="preserve">将来案</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
+          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細拡張</t>
+          <t xml:space="preserve">患者注文拡張</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
+          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -856,27 +856,27 @@
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済接続</t>
+          <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">患者注文明細拡張</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections</t>
+          <t xml:space="preserve">patient_order_items</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">既存テーブル拡張案</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
+          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -888,17 +888,17 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">配送開始</t>
+          <t xml:space="preserve">決済接続</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments</t>
+          <t xml:space="preserve">order_transaction_projections</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
+          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">patient_fulfillments</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
+          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -952,17 +952,17 @@
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入接続</t>
+          <t xml:space="preserve">配送開始</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
+          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入明細</t>
+          <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_items</t>
+          <t xml:space="preserve">patient_subscriptions</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
+          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1016,17 +1016,17 @@
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">定期購入接続</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部受信イベント</t>
+          <t xml:space="preserve">定期購入明細</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">patient_subscription_items</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1053,57 +1053,89 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">外部受信イベント</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shopify接続</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">外部送信キュー</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">将来案</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部APIへ送る処理を永続化するOutbox。</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">別ドメイン</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">医院仕入注文</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">clinic_orders</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">実装済み</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">BGJから医院へのB2B仕入・売上履歴</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文系列へ統合しない</t>
         </is>
@@ -1114,7 +1146,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <autoFilter ref="A4:F22"/>
+  <autoFilter ref="A4:F23"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -1122,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3554,22 +3586,22 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">送り先ID</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_id</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -3579,7 +3611,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK / FK</t>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -3589,12 +3621,12 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr">
@@ -3611,22 +3643,22 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">郵便番号</t>
+          <t xml:space="preserve">医院得意先コード</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">postal_code</t>
+          <t xml:space="preserve">clinic_customer_code</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3634,14 +3666,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -3651,7 +3683,7 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">^[0-9]{3}-[0-9]{4}$</t>
+          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
@@ -3668,37 +3700,37 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">都道府県</t>
+          <t xml:space="preserve">患者ID</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">prefecture</t>
+          <t xml:space="preserve">patient_id</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3708,7 +3740,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2〜4文字</t>
+          <t xml:space="preserve">patients.id ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
@@ -3725,22 +3757,22 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">市区町村</t>
+          <t xml:space="preserve">送り先名</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">city</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3765,7 +3797,7 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜100文字</t>
+          <t xml:space="preserve">1〜50文字</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -3782,22 +3814,22 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所1</t>
+          <t xml:space="preserve">郵便番号</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line1</t>
+          <t xml:space="preserve">postal_code</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -3822,7 +3854,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜200文字</t>
+          <t xml:space="preserve">^[0-9]{3}-[0-9]{4}$</t>
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr">
@@ -3839,22 +3871,22 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所2</t>
+          <t xml:space="preserve">都道府県</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line2</t>
+          <t xml:space="preserve">prefecture</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3869,7 +3901,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -3879,7 +3911,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">200文字以内</t>
+          <t xml:space="preserve">2〜4文字</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
@@ -3896,22 +3928,22 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取人名</t>
+          <t xml:space="preserve">市区町村</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">recipient_name</t>
+          <t xml:space="preserve">city</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -3953,22 +3985,22 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">電話番号</t>
+          <t xml:space="preserve">住所1</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">phone</t>
+          <t xml:space="preserve">address_line1</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3993,7 +4025,7 @@
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字10〜15桁</t>
+          <t xml:space="preserve">1〜200文字</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
@@ -4010,27 +4042,27 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">住所2</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">address_line2</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -4040,17 +4072,17 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">200文字以内</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
@@ -4067,32 +4099,32 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベントID</t>
+          <t xml:space="preserve">受取人名</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">recipient_name</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -4102,12 +4134,12 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1〜100文字</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
@@ -4124,32 +4156,32 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">電話番号</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_id</t>
+          <t xml:space="preserve">phone</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -4164,7 +4196,7 @@
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+          <t xml:space="preserve">数字10〜15桁</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
@@ -4181,27 +4213,27 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベント種別</t>
+          <t xml:space="preserve">既定</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">event_type</t>
+          <t xml:space="preserve">is_default</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">boolean</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -4216,7 +4248,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">false</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -4238,27 +4270,27 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者種別</t>
+          <t xml:space="preserve">削除日時</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_type</t>
+          <t xml:space="preserve">deleted_at</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -4268,7 +4300,7 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
@@ -4295,27 +4327,27 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者識別子</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_identifier</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -4330,7 +4362,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -4352,27 +4384,27 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">変更前状態</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">from_status</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -4382,12 +4414,12 @@
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
@@ -4409,37 +4441,37 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">order_delivery_destinations</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">変更後状態</t>
+          <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">to_status</t>
+          <t xml:space="preserve">order_id</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK / FK</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -4449,7 +4481,7 @@
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr">
@@ -4466,50 +4498,1019 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先ID</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destination_id</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.id ON DELETE RESTRICT</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先名</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">label</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">郵便番号</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">postal_code</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">都道府県</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prefecture</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">市区町村</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">住所1</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">address_line1</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">住所2</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">address_line2</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取人名</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">recipient_name</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">電話番号</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phone</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">作成日時</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">created_at</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_order_events</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベントID</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">内部注文ID</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_id</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベント種別</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">event_type</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者種別</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_type</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者識別子</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_identifier</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">変更前状態</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from_status</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">変更後状態</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to_status</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">発生日時</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">created_at</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">NO</t>
         </is>
       </c>
-      <c r="I62" s="4" t="inlineStr">
+      <c r="I79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">now()</t>
         </is>
       </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K62" s="4" t="inlineStr">
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4520,7 +5521,7 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <autoFilter ref="A4:K62"/>
+  <autoFilter ref="A4:K79"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -9245,7 +10246,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -9467,96 +10468,96 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK1</t>
+          <t xml:space="preserve">UK3</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">provider, external_account_id</t>
+          <t xml:space="preserve">clinic_customer_code WHERE is_default AND deleted_at IS NULL</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">PARTIAL UNIQUE</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部接続先の重複防止。</t>
+          <t xml:space="preserve">医院ごとの有効な既定送り先を1件に限定。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK2</t>
+          <t xml:space="preserve">UK4</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">fulfillment_id, order_item_id</t>
+          <t xml:space="preserve">patient_id WHERE is_default AND deleted_at IS NULL</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">PARTIAL UNIQUE</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一配送への明細重複防止。</t>
+          <t xml:space="preserve">患者ごとの有効な既定送り先を1件に限定。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK3</t>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IDX4</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">order_delivery_destinations</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
+          <t xml:space="preserve">delivery_destination_id</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">INDEX</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部契約の重複防止。</t>
+          <t xml:space="preserve">使用中送り先の削除可否判定。</t>
         </is>
       </c>
     </row>
@@ -9568,17 +10569,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK4</t>
+          <t xml:space="preserve">UK1</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_event_id</t>
+          <t xml:space="preserve">provider, external_account_id</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -9588,7 +10589,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook重複配信の無害化。</t>
+          <t xml:space="preserve">外部接続先の重複防止。</t>
         </is>
       </c>
     </row>
@@ -9600,17 +10601,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK5</t>
+          <t xml:space="preserve">UK2</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_order_id</t>
+          <t xml:space="preserve">fulfillment_id, order_item_id</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -9620,7 +10621,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
+          <t xml:space="preserve">同一配送への明細重複防止。</t>
         </is>
       </c>
     </row>
@@ -9632,273 +10633,258 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">UK3</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部契約の重複防止。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK4</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_event_id</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook重複配信の無害化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK5</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_order_id</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">UK6</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">idempotency_key</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">UNIQUE</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部送信コマンドの二重実行防止。</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">現行リレーション</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親DB日本語名</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親KEY</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親多重度</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子多重度</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子FK</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子DB日本語名</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">削除・備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinics.customer_code</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.customer_code</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patients.id</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.patient_id</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK・現状CASCADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.id</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_order_items.order_id</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文明細</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.customer_code</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.id</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0..1</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">order_shipping_addresses.order_id</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">注文配送先</t>
-        </is>
-      </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.patient_id</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.id</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_order_events.order_id</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">注文操作履歴</t>
-        </is>
-      </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・現状CASCADE</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">商品</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">products.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -9908,7 +10894,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.product_id</t>
+          <t xml:space="preserve">patient_order_items.order_id</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -9918,51 +10904,118 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・SET NULL</t>
+          <t xml:space="preserve">FK・CASCADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将来リレーション案</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.patient_id</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親DB日本語名</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親KEY</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親多重度</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子多重度</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子FK</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子DB日本語名</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">削除・備考</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.id</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
@@ -9984,22 +11037,22 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections.order_id</t>
+          <t xml:space="preserve">order_delivery_destinations.order_id</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -10026,34 +11079,34 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.order_id</t>
+          <t xml:space="preserve">patient_order_events.order_id</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">商品</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.id</t>
+          <t xml:space="preserve">products.id</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -10063,140 +11116,73 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
+          <t xml:space="preserve">patient_order_items.product_id</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">注文明細</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_order_items.id</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">受取配送明細</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・SET NULL</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部コマース接続</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.commerce_account_id</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来リレーション案</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部コマース接続</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部受信イベント</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親DB日本語名</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親KEY</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親多重度</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子多重度</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子FK</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子DB日本語名</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">削除・備考</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -10211,12 +11197,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
+          <t xml:space="preserve">order_transaction_projections.order_id</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部送信キュー</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -10228,12 +11214,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -10248,12 +11234,12 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+          <t xml:space="preserve">patient_fulfillments.order_id</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -10265,12 +11251,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.id</t>
+          <t xml:space="preserve">patient_fulfillments.id</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -10285,12 +11271,12 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
+          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入明細</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -10302,35 +11288,257 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">注文明細</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_items.id</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取配送明細</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者注文</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部受信イベント</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部送信キュー</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_subscriptions.id</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">定期購入明細</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.id</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">0..1</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.subscription_id</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
@@ -10340,8 +11548,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A32:H32"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
@@ -10350,7 +11558,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -10878,528 +12086,749 @@
       </c>
     </row>
     <row r="29" ht="23" customHeight="1">
-      <c r="B29" s="9" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ
+delivery_destinations</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">注文配送先
-order_shipping_addresses</t>
-        </is>
-      </c>
-      <c r="K29" s="9" t="inlineStr">
+order_delivery_destinations</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">日本語項目</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">物理カラム</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KEY</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">日本語項目</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">物理カラム</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先ID</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">内部注文ID</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_id</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK/FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院得意先コード</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_customer_code</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先ID</t>
+        </is>
+      </c>
+      <c r="L33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destination_id</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者ID</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_id</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先名</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">label</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先名</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">label</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">郵便番号</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">postal_code</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">既定</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">is_default</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">住所1</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">address_line1</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">削除日時</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deleted_at</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取人名</t>
+        </is>
+      </c>
+      <c r="L37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">recipient_name</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="23" customHeight="1">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">注文操作履歴
 patient_order_events</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="46">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">日本語項目</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">物理カラム</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">KEY</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">日本語項目</t>
-        </is>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">物理カラム</t>
-        </is>
-      </c>
-      <c r="O31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="11" t="inlineStr">
+    </row>
+    <row r="47">
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベントID</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="F48" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">order_id</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK/FK</t>
-        </is>
-      </c>
-      <c r="K32" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">イベントID</t>
-        </is>
-      </c>
-      <c r="M32" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">郵便番号</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">postal_code</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">内部注文ID</t>
-        </is>
-      </c>
-      <c r="M33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">order_id</t>
-        </is>
-      </c>
-      <c r="O33" s="6" t="inlineStr">
+      <c r="J48" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">都道府県</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">prefecture</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K34" s="11" t="inlineStr">
+    <row r="49">
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">イベント種別</t>
         </is>
       </c>
-      <c r="M34" s="11" t="inlineStr">
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">event_type</t>
         </is>
       </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">市区町村</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">city</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K35" s="11" t="inlineStr">
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="F50" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">操作者種別</t>
         </is>
       </c>
-      <c r="M35" s="11" t="inlineStr">
+      <c r="H50" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">actor_type</t>
         </is>
       </c>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">住所1</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">address_line1</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">変更前状態</t>
         </is>
       </c>
-      <c r="M36" s="11" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">from_status</t>
         </is>
       </c>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">受取人名</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">recipient_name</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K37" s="11" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="F52" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">変更後状態</t>
         </is>
       </c>
-      <c r="M37" s="11" t="inlineStr">
+      <c r="H52" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">to_status</t>
         </is>
       </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">電話番号</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">phone</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">リレーション一覧</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親DB</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親KEY</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子FK</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子DB</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">備考</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">医院</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.customer_code</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patients.id</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.patient_id</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="G49" s="4" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・現状CASCADE</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_order_items.order_id</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.patient_id</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">送り先マスタ</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery_destinations.id</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文配送先</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">0..1</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">order_shipping_addresses.order_id</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_delivery_destinations.order_id</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_order_events.order_id</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">商品</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">products.id</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">0..1</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_order_items.product_id</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・SET NULL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="98">
+  <mergeCells count="111">
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A4:E5"/>
@@ -11464,40 +12893,53 @@
     <mergeCell ref="L23:M23"/>
     <mergeCell ref="N23:O23"/>
     <mergeCell ref="L25:Q26"/>
-    <mergeCell ref="B29:F30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="K29:O30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="A29:E30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="J29:N30"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="F44:J45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="H52:I52"/>
     <mergeCell ref="B26:J27"/>
-    <mergeCell ref="A46:Q46"/>
+    <mergeCell ref="A58:Q58"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
@@ -12407,7 +13849,7 @@
       <c r="A46" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">注文配送先
-order_shipping_addresses</t>
+order_delivery_destinations</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
@@ -12520,17 +13962,17 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">郵便番号</t>
+          <t xml:space="preserve">送り先ID</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">postal_code</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery_destination_id</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr">
@@ -12567,12 +14009,12 @@
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所1</t>
+          <t xml:space="preserve">郵便番号</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line1</t>
+          <t xml:space="preserve">postal_code</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -12614,12 +14056,12 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取人名</t>
+          <t xml:space="preserve">住所1</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">recipient_name</t>
+          <t xml:space="preserve">address_line1</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
@@ -13410,17 +14852,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_shipping_addresses</t>
+          <t xml:space="preserve">delivery_destinations / order_delivery_destinations</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">自宅配送を有効化し、注文時点の配送先を保存する。</t>
+          <t xml:space="preserve">医院・患者の複数送り先と注文時スナップショットを運用する。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所なし配送を許可しない。</t>
+          <t xml:space="preserve">進行中注文の送り先は論理削除不可。</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: add clinic subscription pricing
</commit_message>
<xml_diff>
--- a/project_clinic_order_management_db_definition.xlsx
+++ b/project_clinic_order_management_db_definition.xlsx
@@ -679,12 +679,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">実装済み・患者表示価格</t>
+          <t xml:space="preserve">実装済み・患者表示／定期価格</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院×商品の表示設定と医院価格。clinic_priceがNULLならproducts.priceを患者表示価格にする。</t>
+          <t xml:space="preserve">医院×商品の表示設定、医院通常価格、3ヶ月／6ヶ月定期価格。期間別価格がNULLなら医院通常価格を使用する。</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1218,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院価格</t>
+          <t xml:space="preserve">医院通常価格</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -2748,17 +2748,17 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">3ヶ月価格</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">subscription_3_month_price</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">&gt;= 0。NULLは医院通常価格を使用</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
@@ -2795,47 +2795,47 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院商品設定</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">clinic_product_settings</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">6ヶ月価格</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">subscription_6_month_price</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">&gt;= 0。NULLは医院通常価格を使用</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
@@ -2852,32 +2852,32 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院商品設定</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">clinic_product_settings</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">得意先コード</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">customer_code</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK / UK2構成</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2887,12 +2887,12 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -2919,12 +2919,12 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者ID</t>
+          <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_id</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2932,9 +2932,9 @@
           <t xml:space="preserve">uuid</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2944,17 +2944,17 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">本番前にRESTRICT等へ変更予定</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -2976,12 +2976,12 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文区分</t>
+          <t xml:space="preserve">得意先コード</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_type</t>
+          <t xml:space="preserve">customer_code</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2989,9 +2989,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK / UK2構成</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -3001,12 +3001,12 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">one_time</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">one_time / subscription</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -3033,22 +3033,22 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取方法</t>
+          <t xml:space="preserve">患者ID</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">fulfillment_method</t>
+          <t xml:space="preserve">patient_id</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -3058,17 +3058,17 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">pickup</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">pickup / delivery</t>
+          <t xml:space="preserve">patients.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">本番前にRESTRICT等へ変更予定</t>
         </is>
       </c>
     </row>
@@ -3090,12 +3090,12 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務状態</t>
+          <t xml:space="preserve">注文区分</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">order_type</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">received</t>
+          <t xml:space="preserve">one_time</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">received / preparing / ready / shipped / completed / canceled</t>
+          <t xml:space="preserve">one_time / subscription</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
@@ -3147,17 +3147,17 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文日時</t>
+          <t xml:space="preserve">受取方法</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordered_at</t>
+          <t xml:space="preserve">fulfillment_method</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -3172,12 +3172,12 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve">pickup</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pickup / delivery</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
@@ -3204,17 +3204,17 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">次回提供予定日</t>
+          <t xml:space="preserve">医院業務状態</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">next_fulfillment_date</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -3224,17 +3224,17 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">received</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">received / preparing / ready / shipped / completed / canceled</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
@@ -3261,22 +3261,22 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成元</t>
+          <t xml:space="preserve">注文日時</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">source</t>
+          <t xml:space="preserve">ordered_at</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK1構成</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -3286,12 +3286,12 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">internal</t>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">internal / shopify</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -3318,17 +3318,17 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">登録経路</t>
+          <t xml:space="preserve">次回提供予定日</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_via</t>
+          <t xml:space="preserve">next_fulfillment_date</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -3338,17 +3338,17 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal / bgj_portal / shopify</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
@@ -3375,12 +3375,12 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部注文ID</t>
+          <t xml:space="preserve">作成元</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">external_order_id</t>
+          <t xml:space="preserve">source</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3395,17 +3395,17 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">internal</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">internal / shopify</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
@@ -3432,12 +3432,12 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">同期状態</t>
+          <t xml:space="preserve">登録経路</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sync_status</t>
+          <t xml:space="preserve">created_via</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -3457,12 +3457,12 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">local</t>
+          <t xml:space="preserve">clinic_portal</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">local / pending / synced / error</t>
+          <t xml:space="preserve">clinic_portal / bgj_portal / shopify</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -3489,12 +3489,12 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">同期エラー</t>
+          <t xml:space="preserve">外部注文ID</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sync_error</t>
+          <t xml:space="preserve">external_order_id</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3502,9 +3502,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK1構成</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -3546,37 +3546,37 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">冪等キー</t>
+          <t xml:space="preserve">同期状態</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">idempotency_key</t>
+          <t xml:space="preserve">sync_status</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK2構成</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">local</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">local / pending / synced / error</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
@@ -3603,17 +3603,17 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部更新日時</t>
+          <t xml:space="preserve">同期エラー</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">external_updated_at</t>
+          <t xml:space="preserve">sync_error</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3660,32 +3660,32 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">冪等キー</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">idempotency_key</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK2構成</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3717,12 +3717,12 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">外部更新日時</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">external_updated_at</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3737,12 +3737,12 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3764,32 +3764,32 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文明細ID</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
@@ -3821,32 +3821,32 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_id</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3856,12 +3856,12 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">商品ID</t>
+          <t xml:space="preserve">注文明細ID</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">product_id</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -3901,24 +3901,24 @@
           <t xml:space="preserve">uuid</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">products.id ON DELETE SET NULL</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr">
@@ -3945,22 +3945,22 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文時商品名</t>
+          <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">product_name</t>
+          <t xml:space="preserve">order_id</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
@@ -4002,27 +4002,27 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文時単価</t>
+          <t xml:space="preserve">商品ID</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_price</t>
+          <t xml:space="preserve">product_id</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&gt;= 0</t>
+          <t xml:space="preserve">products.id ON DELETE SET NULL</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">
@@ -4059,17 +4059,17 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">数量</t>
+          <t xml:space="preserve">注文時商品名</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">quantity</t>
+          <t xml:space="preserve">product_name</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -4084,12 +4084,12 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&gt; 0</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
@@ -4116,17 +4116,17 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">単位スナップショット</t>
+          <t xml:space="preserve">注文時単価</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_snapshot</t>
+          <t xml:space="preserve">unit_price</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">&gt;= 0</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
@@ -4173,17 +4173,17 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">画像種別スナップショット</t>
+          <t xml:space="preserve">数量</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">image_type_snapshot</t>
+          <t xml:space="preserve">quantity</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -4198,12 +4198,12 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">supplement</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">supplement / yogurt / toothbrush / oral</t>
+          <t xml:space="preserve">&gt; 0</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">画像URLスナップショット</t>
+          <t xml:space="preserve">単位スナップショット</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">image_url_snapshot</t>
+          <t xml:space="preserve">unit_snapshot</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -4287,12 +4287,12 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">用量スナップショット</t>
+          <t xml:space="preserve">画像種別スナップショット</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">daily_amount_snapshot</t>
+          <t xml:space="preserve">image_type_snapshot</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -4307,17 +4307,17 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">supplement</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">supplement / yogurt / toothbrush / oral</t>
         </is>
       </c>
       <c r="K57" s="4" t="inlineStr">
@@ -4344,12 +4344,12 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内容量スナップショット</t>
+          <t xml:space="preserve">画像URLスナップショット</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">volume_snapshot</t>
+          <t xml:space="preserve">image_url_snapshot</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
@@ -4401,12 +4401,12 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注意事項スナップショット</t>
+          <t xml:space="preserve">用量スナップショット</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">caution_snapshot</t>
+          <t xml:space="preserve">daily_amount_snapshot</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -4458,12 +4458,12 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部明細ID</t>
+          <t xml:space="preserve">内容量スナップショット</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">external_line_item_id</t>
+          <t xml:space="preserve">volume_snapshot</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -4515,17 +4515,17 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">注意事項スナップショット</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">caution_snapshot</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -4535,12 +4535,12 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -4562,42 +4562,42 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations</t>
+          <t xml:space="preserve">patient_order_items</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先ID</t>
+          <t xml:space="preserve">外部明細ID</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">external_line_item_id</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr">
@@ -4619,47 +4619,47 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations</t>
+          <t xml:space="preserve">patient_order_items</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院得意先コード</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_customer_code</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr">
@@ -4686,12 +4686,12 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者ID</t>
+          <t xml:space="preserve">送り先ID</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_id</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -4699,24 +4699,24 @@
           <t xml:space="preserve">uuid</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K64" s="4" t="inlineStr">
@@ -4743,12 +4743,12 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先名</t>
+          <t xml:space="preserve">医院得意先コード</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">label</t>
+          <t xml:space="preserve">clinic_customer_code</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4756,14 +4756,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G65" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜50文字</t>
+          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
@@ -4800,27 +4800,27 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">郵便番号</t>
+          <t xml:space="preserve">患者ID</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">postal_code</t>
+          <t xml:space="preserve">patient_id</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G66" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">^[0-9]{3}-[0-9]{4}$</t>
+          <t xml:space="preserve">patients.id ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K66" s="4" t="inlineStr">
@@ -4857,12 +4857,12 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">都道府県</t>
+          <t xml:space="preserve">送り先名</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">prefecture</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2〜4文字</t>
+          <t xml:space="preserve">1〜50文字</t>
         </is>
       </c>
       <c r="K67" s="4" t="inlineStr">
@@ -4914,12 +4914,12 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">市区町村</t>
+          <t xml:space="preserve">郵便番号</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">city</t>
+          <t xml:space="preserve">postal_code</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜100文字</t>
+          <t xml:space="preserve">^[0-9]{3}-[0-9]{4}$</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
@@ -4971,12 +4971,12 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所1</t>
+          <t xml:space="preserve">都道府県</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line1</t>
+          <t xml:space="preserve">prefecture</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜200文字</t>
+          <t xml:space="preserve">2〜4文字</t>
         </is>
       </c>
       <c r="K69" s="4" t="inlineStr">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所2</t>
+          <t xml:space="preserve">市区町村</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line2</t>
+          <t xml:space="preserve">city</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -5048,7 +5048,7 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">200文字以内</t>
+          <t xml:space="preserve">1〜100文字</t>
         </is>
       </c>
       <c r="K70" s="4" t="inlineStr">
@@ -5085,12 +5085,12 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取人名</t>
+          <t xml:space="preserve">住所1</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">recipient_name</t>
+          <t xml:space="preserve">address_line1</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1〜100文字</t>
+          <t xml:space="preserve">1〜200文字</t>
         </is>
       </c>
       <c r="K71" s="4" t="inlineStr">
@@ -5142,12 +5142,12 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">電話番号</t>
+          <t xml:space="preserve">住所2</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">phone</t>
+          <t xml:space="preserve">address_line2</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字10〜15桁</t>
+          <t xml:space="preserve">200文字以内</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
@@ -5199,17 +5199,17 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既定</t>
+          <t xml:space="preserve">受取人名</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">is_default</t>
+          <t xml:space="preserve">recipient_name</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolean</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -5224,12 +5224,12 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1〜100文字</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
@@ -5256,17 +5256,17 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">削除日時</t>
+          <t xml:space="preserve">電話番号</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">deleted_at</t>
+          <t xml:space="preserve">phone</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">数字10〜15桁</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
@@ -5313,17 +5313,17 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">既定</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">is_default</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">boolean</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve">false</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -5370,12 +5370,12 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">削除日時</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">deleted_at</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -5390,12 +5390,12 @@
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
@@ -5417,32 +5417,32 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_id</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK / FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -5452,12 +5452,12 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
@@ -5474,32 +5474,32 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations</t>
+          <t xml:space="preserve">delivery_destinations</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先ID</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destination_id</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G78" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -5509,12 +5509,12 @@
       </c>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.id ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
@@ -5541,22 +5541,22 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先名</t>
+          <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">label</t>
+          <t xml:space="preserve">order_id</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK / FK</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -5598,22 +5598,22 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">郵便番号</t>
+          <t xml:space="preserve">送り先ID</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">postal_code</t>
+          <t xml:space="preserve">delivery_destination_id</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery_destinations.id ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -5655,12 +5655,12 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">都道府県</t>
+          <t xml:space="preserve">送り先名</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">prefecture</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">市区町村</t>
+          <t xml:space="preserve">郵便番号</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">city</t>
+          <t xml:space="preserve">postal_code</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
@@ -5769,12 +5769,12 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所1</t>
+          <t xml:space="preserve">都道府県</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line1</t>
+          <t xml:space="preserve">prefecture</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">住所2</t>
+          <t xml:space="preserve">市区町村</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">address_line2</t>
+          <t xml:space="preserve">city</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr">
@@ -5883,12 +5883,12 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取人名</t>
+          <t xml:space="preserve">住所1</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">recipient_name</t>
+          <t xml:space="preserve">address_line1</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
@@ -5940,12 +5940,12 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">電話番号</t>
+          <t xml:space="preserve">住所2</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">phone</t>
+          <t xml:space="preserve">address_line2</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
@@ -5997,17 +5997,17 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">受取人名</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">recipient_name</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
@@ -6044,32 +6044,32 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">order_delivery_destinations</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベントID</t>
+          <t xml:space="preserve">電話番号</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">phone</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
@@ -6079,7 +6079,7 @@
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
@@ -6101,32 +6101,32 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events</t>
+          <t xml:space="preserve">order_delivery_destinations</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">内部注文ID</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_id</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G89" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -6136,12 +6136,12 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
@@ -6168,22 +6168,22 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベント種別</t>
+          <t xml:space="preserve">イベントID</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">event_type</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G90" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr">
@@ -6225,22 +6225,22 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者種別</t>
+          <t xml:space="preserve">内部注文ID</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_type</t>
+          <t xml:space="preserve">order_id</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G91" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">patient_orders.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
@@ -6282,12 +6282,12 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者識別子</t>
+          <t xml:space="preserve">イベント種別</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_identifier</t>
+          <t xml:space="preserve">event_type</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
@@ -6339,12 +6339,12 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">変更前状態</t>
+          <t xml:space="preserve">操作者種別</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">from_status</t>
+          <t xml:space="preserve">actor_type</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
@@ -6396,12 +6396,12 @@
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">変更後状態</t>
+          <t xml:space="preserve">操作者識別子</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">to_status</t>
+          <t xml:space="preserve">actor_identifier</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
@@ -6453,40 +6453,154 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">変更前状態</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from_status</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="30" customHeight="1">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">変更後状態</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to_status</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文操作履歴</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_events</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">発生日時</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
+      <c r="E97" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">created_at</t>
         </is>
       </c>
-      <c r="F95" s="4" t="inlineStr">
+      <c r="F97" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">NO</t>
         </is>
       </c>
-      <c r="I95" s="4" t="inlineStr">
+      <c r="I97" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">now()</t>
         </is>
       </c>
-      <c r="J95" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K95" s="4" t="inlineStr">
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6497,7 +6611,7 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <autoFilter ref="A4:K95"/>
+  <autoFilter ref="A4:K97"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -13682,7 +13796,7 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院価格</t>
+          <t xml:space="preserve">医院通常価格</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
@@ -13691,6 +13805,40 @@
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3ヶ月価格</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subscription_3_month_price</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6ヶ月価格</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subscription_6_month_price</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -14185,7 +14333,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="131">
+  <mergeCells count="135">
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A4:E5"/>
@@ -14315,6 +14463,10 @@
     <mergeCell ref="C63:D63"/>
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="C64:D64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="C66:D66"/>
     <mergeCell ref="B26:J27"/>
     <mergeCell ref="A72:Q72"/>
   </mergeCells>
@@ -16266,12 +16418,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院価格と注文時商品画像を運用する。</t>
+          <t xml:space="preserve">医院通常・期間別価格と注文時商品画像を運用する。</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">仕切値は導出し、重複保存しない。</t>
+          <t xml:space="preserve">仕切値と価格既定値は重複保存しない。</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: centralize clinic contact and login management
</commit_message>
<xml_diff>
--- a/project_clinic_order_management_db_definition.xlsx
+++ b/project_clinic_order_management_db_definition.xlsx
@@ -266,7 +266,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院が患者向け商品を管理するpatient_orders系列、およびウェビナー管理</t>
+          <t xml:space="preserve">医院が患者向け商品を管理するpatient_orders系列、ウェビナー、医院業務連絡担当者</t>
         </is>
       </c>
     </row>
@@ -290,7 +290,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Supabaseの患者注文・定期購入申込・送り先・ウェビナー各テーブル</t>
+          <t xml:space="preserve">Supabaseの患者注文・定期購入申込・送り先・ウェビナー・医院担当者各テーブル</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1112,27 +1112,27 @@
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
+          <t xml:space="preserve">医院ごとに複数の業務連絡担当者と主担当、論理削除、排他制御を管理する。</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1144,27 +1144,27 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文拡張</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存テーブル拡張案</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
+          <t xml:space="preserve">担当者ごとの連絡内容と方法を多値属性として分離する。</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1176,27 +1176,27 @@
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細拡張</t>
+          <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items</t>
+          <t xml:space="preserve">clinic_contact_events</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存テーブル拡張案</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
+          <t xml:space="preserve">登録・更新・無効化・主担当変更・論理削除を監査保存する。</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1208,17 +1208,17 @@
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済接続</t>
+          <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
+          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1240,27 +1240,27 @@
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">配送開始</t>
+          <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">患者注文拡張</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">既存テーブル拡張案</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
+          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1272,27 +1272,27 @@
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">配送開始</t>
+          <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">患者注文明細拡張</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">patient_order_items</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">既存テーブル拡張案</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
+          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1304,17 +1304,17 @@
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入接続</t>
+          <t xml:space="preserve">決済接続</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">order_transaction_projections</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
+          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1336,17 +1336,17 @@
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入接続</t>
+          <t xml:space="preserve">配送開始</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入明細</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_items</t>
+          <t xml:space="preserve">patient_fulfillments</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
+          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1368,17 +1368,17 @@
     <row r="31" ht="34" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">配送開始</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部受信イベント</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1400,62 +1400,158 @@
     <row r="32" ht="34" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">定期購入接続</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">定期購入接続</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">定期購入明細</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_items</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部受信イベント</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shopify接続</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部送信キュー</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">将来案</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部APIへ送る処理を永続化するOutbox。</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">別ドメイン</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">医院仕入注文</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">clinic_orders</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">実装済み</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">BGJから医院へのB2B仕入・売上履歴</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文系列へ統合しない</t>
         </is>
@@ -1466,7 +1562,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <autoFilter ref="A4:F33"/>
+  <autoFilter ref="A4:F36"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -1474,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K169"/>
+  <dimension ref="A1:K196"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -10966,12 +11062,1551 @@
         </is>
       </c>
     </row>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者ID</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="J170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">得意先コード</t>
+        </is>
+      </c>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">customer_code</t>
+        </is>
+      </c>
+      <c r="F171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G171" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
+        </is>
+      </c>
+      <c r="K171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="30" customHeight="1">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院ログインID</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_user_id</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G172" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_users.id ON DELETE SET NULL</t>
+        </is>
+      </c>
+      <c r="K172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="30" customHeight="1">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">氏名</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="F173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="30" customHeight="1">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部署</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">department</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="30" customHeight="1">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">役職</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">title</t>
+        </is>
+      </c>
+      <c r="F175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="30" customHeight="1">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">メールアドレス</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">email</t>
+        </is>
+      </c>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="30" customHeight="1">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">電話番号</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phone</t>
+        </is>
+      </c>
+      <c r="F177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="30" customHeight="1">
+      <c r="A178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主担当</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">is_primary</t>
+        </is>
+      </c>
+      <c r="F178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">boolean</t>
+        </is>
+      </c>
+      <c r="G178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="30" customHeight="1">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">状態</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="F179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active / inactive</t>
+        </is>
+      </c>
+      <c r="K179" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">備考</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">排他バージョン</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">version</t>
+        </is>
+      </c>
+      <c r="F181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">論理削除日時</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deleted_at</t>
+        </is>
+      </c>
+      <c r="F182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">作成日時</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">created_at</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">更新日時</t>
+        </is>
+      </c>
+      <c r="E184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">updated_at</t>
+        </is>
+      </c>
+      <c r="F184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者ID</t>
+        </is>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">contact_id</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK / FK</t>
+        </is>
+      </c>
+      <c r="H185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
+        </is>
+      </c>
+      <c r="K185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通知種別</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">topic</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">webinar / orders / billing / product / system / sales</t>
+        </is>
+      </c>
+      <c r="K186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">連絡方法</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">channel</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">email / phone</t>
+        </is>
+      </c>
+      <c r="K187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="30" customHeight="1">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">有効</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">enabled</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">boolean</t>
+        </is>
+      </c>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="J188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="30" customHeight="1">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">作成日時</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">created_at</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="30" customHeight="1">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">更新日時</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">updated_at</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベントID</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="J191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="30" customHeight="1">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者ID</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">contact_id</t>
+        </is>
+      </c>
+      <c r="F192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G192" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
+        </is>
+      </c>
+      <c r="K192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="30" customHeight="1">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベント種別</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">event_type</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="30" customHeight="1">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者種別</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_type</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="30" customHeight="1">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者識別子</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_identifier</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">発生日時</t>
+        </is>
+      </c>
+      <c r="E196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">created_at</t>
+        </is>
+      </c>
+      <c r="F196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">now()</t>
+        </is>
+      </c>
+      <c r="J196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <autoFilter ref="A4:K169"/>
+  <autoFilter ref="A4:K196"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -15696,7 +17331,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -16238,96 +17873,96 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK1</t>
+          <t xml:space="preserve">UK10</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">provider, external_account_id</t>
+          <t xml:space="preserve">customer_code WHERE is_primary AND status='active' AND deleted_at IS NULL</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">PARTIAL UNIQUE</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部接続先の重複防止。</t>
+          <t xml:space="preserve">医院ごとの有効な主担当を1人に限定。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK2</t>
+          <t xml:space="preserve">UK11</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">fulfillment_id, order_item_id</t>
+          <t xml:space="preserve">customer_code, lower(email) WHERE deleted_at IS NULL</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">PARTIAL UNIQUE</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一配送への明細重複防止。</t>
+          <t xml:space="preserve">医院内の担当者メール重複防止。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK3</t>
+          <t xml:space="preserve">UK12</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
+          <t xml:space="preserve">clinic_user_id WHERE deleted_at IS NULL</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNIQUE</t>
+          <t xml:space="preserve">PARTIAL UNIQUE</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部契約の重複防止。</t>
+          <t xml:space="preserve">1ログインと複数担当者の誤関連防止。</t>
         </is>
       </c>
     </row>
@@ -16339,17 +17974,17 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK4</t>
+          <t xml:space="preserve">UK1</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_event_id</t>
+          <t xml:space="preserve">provider, external_account_id</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -16359,7 +17994,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook重複配信の無害化。</t>
+          <t xml:space="preserve">外部接続先の重複防止。</t>
         </is>
       </c>
     </row>
@@ -16371,17 +18006,17 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK5</t>
+          <t xml:space="preserve">UK2</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_order_id</t>
+          <t xml:space="preserve">fulfillment_id, order_item_id</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -16391,7 +18026,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
+          <t xml:space="preserve">同一配送への明細重複防止。</t>
         </is>
       </c>
     </row>
@@ -16403,182 +18038,167 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">UK3</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部契約の重複防止。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK4</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_event_id</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook重複配信の無害化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK5</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_account_id, external_order_id</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIQUE</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">UK6</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">idempotency_key</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">UNIQUE</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部送信コマンドの二重実行防止。</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">現行リレーション</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親DB日本語名</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親KEY</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親多重度</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子多重度</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子FK</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子DB日本語名</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">削除・備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinics.customer_code</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0..1</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_terms.customer_code</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院契約情報</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinics.customer_code</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_product_settings.customer_code</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院商品設定</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">商品</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">products.id</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_product_settings.product_id</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院商品設定</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -16600,34 +18220,34 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.customer_code</t>
+          <t xml:space="preserve">clinic_terms.customer_code</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院契約情報</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -16642,29 +18262,29 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.patient_id</t>
+          <t xml:space="preserve">clinic_product_settings.customer_code</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院商品設定</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・現状CASCADE</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">商品</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">products.id</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -16679,17 +18299,17 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.order_id</t>
+          <t xml:space="preserve">clinic_product_settings.product_id</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">医院商品設定</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -16716,17 +18336,17 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
+          <t xml:space="preserve">patient_orders.customer_code</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
@@ -16753,29 +18373,29 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.patient_id</t>
+          <t xml:space="preserve">patient_orders.patient_id</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・現状CASCADE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -16790,29 +18410,29 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
+          <t xml:space="preserve">patient_order_items.order_id</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -16822,34 +18442,34 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations.order_id</t>
+          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">患者</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">patients.id</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -16864,34 +18484,34 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events.order_id</t>
+          <t xml:space="preserve">delivery_destinations.patient_id</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">商品</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">products.id</t>
+          <t xml:space="preserve">delivery_destinations.id</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -16901,29 +18521,29 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.product_id</t>
+          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・SET NULL</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -16933,34 +18553,34 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.customer_code</t>
+          <t xml:space="preserve">order_delivery_destinations.order_id</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -16975,34 +18595,34 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.patient_id</t>
+          <t xml:space="preserve">patient_order_events.order_id</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">商品</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.id</t>
+          <t xml:space="preserve">products.id</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -17012,103 +18632,103 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_items.request_id</t>
+          <t xml:space="preserve">patient_order_items.product_id</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込明細</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・SET NULL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_requests.customer_code</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_requests.id</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0..1</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_request_destinations.request_id</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">定期購入申込配送先</t>
-        </is>
-      </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_requests.patient_id</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_requests.id</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_request_events.request_id</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">定期購入申込履歴</t>
-        </is>
-      </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.id</t>
+          <t xml:space="preserve">patient_subscription_requests.id</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -17123,29 +18743,29 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_destinations.delivery_destination_id</t>
+          <t xml:space="preserve">patient_subscription_request_items.request_id</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込配送先</t>
+          <t xml:space="preserve">定期購入申込明細</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinars.id</t>
+          <t xml:space="preserve">patient_subscription_requests.id</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -17155,34 +18775,34 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_sessions.webinar_id</t>
+          <t xml:space="preserve">patient_subscription_request_destinations.request_id</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー開催枠</t>
+          <t xml:space="preserve">定期購入申込配送先</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinars.id</t>
+          <t xml:space="preserve">patient_subscription_requests.id</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -17197,29 +18817,29 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_target_clinics.webinar_id</t>
+          <t xml:space="preserve">patient_subscription_request_events.request_id</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー対象医院</t>
+          <t xml:space="preserve">定期購入申込履歴</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">delivery_destinations.id</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -17234,17 +18854,17 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_target_clinics.customer_code</t>
+          <t xml:space="preserve">patient_subscription_request_destinations.delivery_destination_id</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー対象医院</t>
+          <t xml:space="preserve">定期購入申込配送先</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
@@ -17271,73 +18891,140 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">webinar_sessions.webinar_id</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ウェビナー開催枠</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・CASCADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ウェビナー</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">webinars.id</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">webinar_target_clinics.webinar_id</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ウェビナー対象医院</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">webinar_target_clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ウェビナー対象医院</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ウェビナー</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">webinars.id</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">webinar_events.webinar_id</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">ウェビナー操作履歴</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・CASCADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将来リレーション案</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親DB日本語名</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親KEY</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親多重度</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子多重度</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子FK</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子DB日本語名</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">削除・備考</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -17352,29 +19039,29 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections.order_id</t>
+          <t xml:space="preserve">clinic_contacts.customer_code</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院ログイン</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">clinic_users.id</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -17384,34 +19071,34 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.order_id</t>
+          <t xml:space="preserve">clinic_contacts.clinic_user_id</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・SET NULL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.id</t>
+          <t xml:space="preserve">clinic_contacts.id</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -17426,29 +19113,29 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文明細</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.id</t>
+          <t xml:space="preserve">clinic_contacts.id</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -17463,140 +19150,73 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
+          <t xml:space="preserve">clinic_contact_events.contact_id</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部コマース接続</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.commerce_account_id</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部コマース接続</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部受信イベント</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来リレーション案</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部コマース接続</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部送信キュー</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親DB日本語名</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親KEY</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親多重度</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子多重度</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子FK</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子DB日本語名</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">削除・備考</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -17611,12 +19231,12 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+          <t xml:space="preserve">order_transaction_projections.order_id</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -17628,12 +19248,12 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -17648,12 +19268,12 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
+          <t xml:space="preserve">patient_fulfillments.order_id</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入明細</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -17665,35 +19285,294 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">受取配送</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillments.id</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取配送明細</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注文明細</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_order_items.id</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取配送明細</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者注文</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部受信イベント</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部コマース接続</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_accounts.id</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">外部送信キュー</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_subscriptions.id</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">定期購入明細</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.id</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">0..1</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.subscription_id</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
@@ -17703,8 +19582,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A59:H59"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
@@ -17713,7 +19592,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q95"/>
+  <dimension ref="A1:Q99"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -19653,6 +21532,154 @@
       <c r="G95" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・CASCADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.customer_code</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院ログイン</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_users.id</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0..1</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.clinic_user_id</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・SET NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events.contact_id</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: unify clinic contacts with login identities
</commit_message>
<xml_diff>
--- a/project_clinic_order_management_db_definition.xlsx
+++ b/project_clinic_order_management_db_definition.xlsx
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ごとに複数の業務連絡担当者と主担当、論理削除、排他制御を管理する。</t>
+          <t xml:space="preserve">医院担当者の役職を選択肢として一元管理する。</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1149,22 +1149,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">実装済み・Phase 1</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">認証情報とセッション世代を保持する。担当者プロフィールとはclinic_contactsで関連する。</t>
+          <t xml:space="preserve">医院ごとに複数の業務連絡担当者と主担当、論理削除、排他制御を管理する。</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">管理者・一般・閲覧専用の権限マスタ。</t>
+          <t xml:space="preserve">担当者ID・認証情報・所属得意先・セッション世代を保持する。全担当者が1対1でclinic_contactsを持つ。</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限機能</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限と操作可能な機能を多対多で管理する。</t>
+          <t xml:space="preserve">管理者・一般・閲覧専用の権限マスタ。</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限機能</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_role_permissions</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1ログインに1権限を割り当て、認証情報と権限マスタを分離する。</t>
+          <t xml:space="preserve">権限と操作可能な機能を多対多で管理する。</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1277,22 +1277,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">実装済み</t>
+          <t xml:space="preserve">実装済み・Phase 1</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者ごとの連絡内容と方法を多値属性として分離する。</t>
+          <t xml:space="preserve">1ログインに1権限を割り当て、認証情報と権限マスタを分離する。</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">登録・更新・無効化・主担当変更・論理削除を監査保存する。</t>
+          <t xml:space="preserve">担当者ごとの連絡内容と方法を多値属性として分離する。</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1336,27 +1336,27 @@
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">現行</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">clinic_contact_events</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">実装済み</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
+          <t xml:space="preserve">登録・更新・無効化・主担当変更・論理削除を監査保存する。</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1373,22 +1373,22 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文拡張</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存テーブル拡張案</t>
+          <t xml:space="preserve">将来案</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
+          <t xml:space="preserve">Shopifyストア等の外部接続先。医院との対応方式は接続構成確定後に決定する。</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細拡張</t>
+          <t xml:space="preserve">患者注文拡張</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
+          <t xml:space="preserve">既存IDを維持し、外部・金額・排他制御の列を追加する。</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1432,27 +1432,27 @@
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済接続</t>
+          <t xml:space="preserve">Shopify接続</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">患者注文明細拡張</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections</t>
+          <t xml:space="preserve">patient_order_items</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">将来案</t>
+          <t xml:space="preserve">既存テーブル拡張案</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
+          <t xml:space="preserve">外部明細と通貨を明確化し、既存スナップショットを維持する。</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -1464,17 +1464,17 @@
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">配送開始</t>
+          <t xml:space="preserve">決済接続</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments</t>
+          <t xml:space="preserve">order_transaction_projections</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
+          <t xml:space="preserve">Shopify上の決済・返金を表示する投影。会計台帳ではない。</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">patient_fulfillments</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
+          <t xml:space="preserve">医院受け取り・配送・部分引き渡しの単位。</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -1528,17 +1528,17 @@
     <row r="36" ht="34" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入接続</t>
+          <t xml:space="preserve">配送開始</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
+          <t xml:space="preserve">部分受け取り・部分配送時の対象明細と数量。</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入明細</t>
+          <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_items</t>
+          <t xml:space="preserve">patient_subscriptions</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
+          <t xml:space="preserve">Shopify上の定期購入契約を患者ポータルへ表示する投影。</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1592,17 +1592,17 @@
     <row r="38" ht="34" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify接続</t>
+          <t xml:space="preserve">定期購入接続</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部受信イベント</t>
+          <t xml:space="preserve">定期購入明細</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">patient_subscription_items</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+          <t xml:space="preserve">契約時点の商品・数量・単価の投影。</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1629,57 +1629,89 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">外部受信イベント</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commerce_webhook_events</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来案</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhookを先に永続化し、重複排除・再試行するInbox。</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shopify接続</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">外部送信キュー</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">将来案</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">外部APIへ送る処理を永続化するOutbox。</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">別ドメイン</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">医院仕入注文</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">clinic_orders</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">実装済み</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">BGJから医院へのB2B仕入・売上履歴</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文系列へ統合しない</t>
         </is>
@@ -1690,7 +1722,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <autoFilter ref="A4:F40"/>
+  <autoFilter ref="A4:F41"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -1698,7 +1730,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K225"/>
+  <dimension ref="A1:K231"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -11198,27 +11230,27 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者ID</t>
+          <t xml:space="preserve">役職キー</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">role_key</t>
         </is>
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G170" s="5" t="inlineStr">
@@ -11233,12 +11265,12 @@
       </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">physician / dentist / nurse / dental_hygienist / receptionist / other</t>
         </is>
       </c>
       <c r="K170" s="4" t="inlineStr">
@@ -11255,22 +11287,22 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">得意先コード</t>
+          <t xml:space="preserve">役職名</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">customer_code</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="F171" s="4" t="inlineStr">
@@ -11278,9 +11310,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G171" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+      <c r="G171" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr">
@@ -11295,7 +11327,7 @@
       </c>
       <c r="J171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K171" s="4" t="inlineStr">
@@ -11312,37 +11344,37 @@
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログインID</t>
+          <t xml:space="preserve">表示順</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_id</t>
+          <t xml:space="preserve">sort_order</t>
         </is>
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G172" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G172" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK</t>
         </is>
       </c>
       <c r="H172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
@@ -11352,7 +11384,7 @@
       </c>
       <c r="J172" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id ON DELETE SET NULL</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K172" s="4" t="inlineStr">
@@ -11369,27 +11401,27 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">氏名</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -11404,7 +11436,7 @@
       </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J173" s="4" t="inlineStr">
@@ -11426,27 +11458,27 @@
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_contact_roles</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">部署</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">department</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -11456,12 +11488,12 @@
       </c>
       <c r="H174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J174" s="4" t="inlineStr">
@@ -11493,32 +11525,32 @@
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">役職</t>
+          <t xml:space="preserve">担当者ID</t>
         </is>
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">title</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G175" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G175" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J175" s="4" t="inlineStr">
@@ -11550,12 +11582,12 @@
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">メールアドレス</t>
+          <t xml:space="preserve">得意先コード</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">customer_code</t>
         </is>
       </c>
       <c r="F176" s="4" t="inlineStr">
@@ -11563,14 +11595,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G176" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G176" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr">
@@ -11580,7 +11612,7 @@
       </c>
       <c r="J176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">clinics.customer_code ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K176" s="4" t="inlineStr">
@@ -11607,27 +11639,27 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">電話番号</t>
+          <t xml:space="preserve">認証アカウント内部ID</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">phone</t>
+          <t xml:space="preserve">clinic_user_id</t>
         </is>
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G177" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G177" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK / FK</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I177" s="4" t="inlineStr">
@@ -11637,7 +11669,7 @@
       </c>
       <c r="J177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">clinic_users.(id, customer_code) ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K177" s="4" t="inlineStr">
@@ -11664,17 +11696,17 @@
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">主担当</t>
+          <t xml:space="preserve">氏名</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">is_primary</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolean</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -11689,7 +11721,7 @@
       </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J178" s="4" t="inlineStr">
@@ -11721,12 +11753,12 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">状態</t>
+          <t xml:space="preserve">部署</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">department</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr">
@@ -11741,17 +11773,17 @@
       </c>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">active</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">active / inactive</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K179" s="4" t="inlineStr">
@@ -11778,12 +11810,12 @@
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">備考</t>
+          <t xml:space="preserve">役職キー</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">notes</t>
+          <t xml:space="preserve">role_key</t>
         </is>
       </c>
       <c r="F180" s="4" t="inlineStr">
@@ -11791,24 +11823,24 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G180" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G180" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">other</t>
         </is>
       </c>
       <c r="J180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">clinic_contact_roles.role_key ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K180" s="4" t="inlineStr">
@@ -11835,17 +11867,17 @@
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">排他バージョン</t>
+          <t xml:space="preserve">メールアドレス</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">version</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -11855,12 +11887,12 @@
       </c>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J181" s="4" t="inlineStr">
@@ -11892,17 +11924,17 @@
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">論理削除日時</t>
+          <t xml:space="preserve">電話番号</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">deleted_at</t>
+          <t xml:space="preserve">phone</t>
         </is>
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -11949,17 +11981,17 @@
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">主担当</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">is_primary</t>
         </is>
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">boolean</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -11974,7 +12006,7 @@
       </c>
       <c r="I183" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve">false</t>
         </is>
       </c>
       <c r="J183" s="4" t="inlineStr">
@@ -12006,17 +12038,17 @@
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">状態</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -12031,12 +12063,12 @@
       </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve">active</t>
         </is>
       </c>
       <c r="J184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">active / inactive</t>
         </is>
       </c>
       <c r="K184" s="4" t="inlineStr">
@@ -12053,42 +12085,42 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログインID</t>
+          <t xml:space="preserve">備考</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">notes</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G185" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J185" s="4" t="inlineStr">
@@ -12110,32 +12142,32 @@
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">得意先コード</t>
+          <t xml:space="preserve">排他バージョン</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">customer_code</t>
+          <t xml:space="preserve">version</t>
         </is>
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G186" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H186" s="4" t="inlineStr">
@@ -12145,12 +12177,12 @@
       </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K186" s="4" t="inlineStr">
@@ -12167,37 +12199,37 @@
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ログインID</t>
+          <t xml:space="preserve">論理削除日時</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">login_id</t>
+          <t xml:space="preserve">deleted_at</t>
         </is>
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G187" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I187" s="4" t="inlineStr">
@@ -12224,27 +12256,27 @@
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">パスワードハッシュ</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">password_hash</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -12259,7 +12291,7 @@
       </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J188" s="4" t="inlineStr">
@@ -12281,27 +12313,27 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">clinic_contacts</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">表示名</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -12311,12 +12343,12 @@
       </c>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J189" s="4" t="inlineStr">
@@ -12348,32 +12380,32 @@
       </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">メールアドレス</t>
+          <t xml:space="preserve">医院ログインID</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G190" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">gen_random_uuid()</t>
         </is>
       </c>
       <c r="J190" s="4" t="inlineStr">
@@ -12405,12 +12437,12 @@
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">状態</t>
+          <t xml:space="preserve">得意先コード</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">customer_code</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr">
@@ -12418,9 +12450,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G191" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G191" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H191" s="4" t="inlineStr">
@@ -12430,12 +12462,12 @@
       </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">有効</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">有効 / 無効</t>
+          <t xml:space="preserve">clinics.customer_code ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K191" s="4" t="inlineStr">
@@ -12462,22 +12494,22 @@
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">担当者ID兼ログインID</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">login_id</t>
         </is>
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
-        </is>
-      </c>
-      <c r="G192" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK</t>
         </is>
       </c>
       <c r="H192" s="4" t="inlineStr">
@@ -12487,7 +12519,7 @@
       </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J192" s="4" t="inlineStr">
@@ -12497,7 +12529,7 @@
       </c>
       <c r="K192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">A+6桁。画面では担当者IDとして表示し、この値でログインする</t>
         </is>
       </c>
     </row>
@@ -12519,17 +12551,17 @@
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">パスワードハッシュ</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">password_hash</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -12544,7 +12576,7 @@
       </c>
       <c r="I193" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J193" s="4" t="inlineStr">
@@ -12576,17 +12608,17 @@
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ログイン失敗回数</t>
+          <t xml:space="preserve">表示名</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">failed_login_attempts</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -12596,12 +12628,12 @@
       </c>
       <c r="H194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J194" s="4" t="inlineStr">
@@ -12633,17 +12665,17 @@
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ロック解除日時</t>
+          <t xml:space="preserve">メールアドレス</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">locked_until</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -12690,17 +12722,17 @@
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">セッション世代</t>
+          <t xml:space="preserve">状態</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">session_version</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -12715,17 +12747,17 @@
       </c>
       <c r="I196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">有効</t>
         </is>
       </c>
       <c r="J196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&gt; 0</t>
+          <t xml:space="preserve">有効 / 無効</t>
         </is>
       </c>
       <c r="K196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">無効化・パスワード変更時に加算し旧セッションを失効</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -12747,12 +12779,12 @@
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">最終ログイン日時</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">last_login_at</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr">
@@ -12767,12 +12799,12 @@
       </c>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I197" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J197" s="4" t="inlineStr">
@@ -12804,12 +12836,12 @@
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">パスワード変更日時</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">password_changed_at</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F198" s="4" t="inlineStr">
@@ -12824,12 +12856,12 @@
       </c>
       <c r="H198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">NO</t>
         </is>
       </c>
       <c r="I198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J198" s="4" t="inlineStr">
@@ -12851,32 +12883,32 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限キー</t>
+          <t xml:space="preserve">ログイン失敗回数</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">role_key</t>
+          <t xml:space="preserve">failed_login_attempts</t>
         </is>
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G199" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H199" s="4" t="inlineStr">
@@ -12886,12 +12918,12 @@
       </c>
       <c r="I199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="J199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin / staff / viewer</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K199" s="4" t="inlineStr">
@@ -12908,37 +12940,37 @@
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限名</t>
+          <t xml:space="preserve">ロック解除日時</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">label</t>
+          <t xml:space="preserve">locked_until</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G200" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G200" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I200" s="4" t="inlineStr">
@@ -12965,27 +12997,27 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">説明</t>
+          <t xml:space="preserve">セッション世代</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">description</t>
+          <t xml:space="preserve">session_version</t>
         </is>
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -13000,17 +13032,17 @@
       </c>
       <c r="I201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">&gt; 0</t>
         </is>
       </c>
       <c r="K201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">無効化・パスワード変更時に加算し旧セッションを失効</t>
         </is>
       </c>
     </row>
@@ -13022,37 +13054,37 @@
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">表示順</t>
+          <t xml:space="preserve">最終ログイン日時</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sort_order</t>
+          <t xml:space="preserve">last_login_at</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="G202" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G202" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I202" s="4" t="inlineStr">
@@ -13079,22 +13111,22 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">パスワード変更日時</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">password_changed_at</t>
         </is>
       </c>
       <c r="F203" s="4" t="inlineStr">
@@ -13109,12 +13141,12 @@
       </c>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">YES</t>
         </is>
       </c>
       <c r="I203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J203" s="4" t="inlineStr">
@@ -13136,27 +13168,27 @@
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">初回変更必須</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">must_change_password</t>
         </is>
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">boolean</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -13171,7 +13203,7 @@
       </c>
       <c r="I204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve">false</t>
         </is>
       </c>
       <c r="J204" s="4" t="inlineStr">
@@ -13181,7 +13213,7 @@
       </c>
       <c r="K204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">新規発行時true。初回変更または既存リセット完了時false</t>
         </is>
       </c>
     </row>
@@ -13193,12 +13225,12 @@
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限機能</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -13218,7 +13250,7 @@
       </c>
       <c r="G205" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK / FK</t>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H205" s="4" t="inlineStr">
@@ -13233,7 +13265,7 @@
       </c>
       <c r="J205" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key ON DELETE RESTRICT</t>
+          <t xml:space="preserve">admin / staff / viewer</t>
         </is>
       </c>
       <c r="K205" s="4" t="inlineStr">
@@ -13250,22 +13282,22 @@
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限機能</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">機能キー</t>
+          <t xml:space="preserve">権限名</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">permission_key</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -13273,9 +13305,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G206" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+      <c r="G206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK</t>
         </is>
       </c>
       <c r="H206" s="4" t="inlineStr">
@@ -13290,7 +13322,7 @@
       </c>
       <c r="J206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">view_contacts / manage_contacts / manage_logins</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K206" s="4" t="inlineStr">
@@ -13307,27 +13339,27 @@
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限機能</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">説明</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">description</t>
         </is>
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -13342,7 +13374,7 @@
       </c>
       <c r="I207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J207" s="4" t="inlineStr">
@@ -13364,32 +13396,32 @@
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログインID</t>
+          <t xml:space="preserve">表示順</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_id</t>
+          <t xml:space="preserve">sort_order</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G208" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK / FK</t>
+          <t xml:space="preserve">integer</t>
+        </is>
+      </c>
+      <c r="G208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK</t>
         </is>
       </c>
       <c r="H208" s="4" t="inlineStr">
@@ -13404,7 +13436,7 @@
       </c>
       <c r="J208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id ON DELETE CASCADE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K208" s="4" t="inlineStr">
@@ -13421,32 +13453,32 @@
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限キー</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">role_key</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G209" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G209" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H209" s="4" t="inlineStr">
@@ -13456,12 +13488,12 @@
       </c>
       <c r="I209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J209" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K209" s="4" t="inlineStr">
@@ -13478,27 +13510,27 @@
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_roles</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">割当操作者</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">assigned_by</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -13513,7 +13545,7 @@
       </c>
       <c r="I210" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">system</t>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J210" s="4" t="inlineStr">
@@ -13535,32 +13567,32 @@
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限機能</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_role_permissions</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">作成日時</t>
+          <t xml:space="preserve">権限キー</t>
         </is>
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">created_at</t>
+          <t xml:space="preserve">role_key</t>
         </is>
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
-        </is>
-      </c>
-      <c r="G211" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK / FK</t>
         </is>
       </c>
       <c r="H211" s="4" t="inlineStr">
@@ -13570,12 +13602,12 @@
       </c>
       <c r="I211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J211" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">clinic_portal_roles.role_key ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K211" s="4" t="inlineStr">
@@ -13592,32 +13624,32 @@
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン権限割当</t>
+          <t xml:space="preserve">医院ポータル権限機能</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments</t>
+          <t xml:space="preserve">clinic_portal_role_permissions</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">更新日時</t>
+          <t xml:space="preserve">機能キー</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">updated_at</t>
+          <t xml:space="preserve">permission_key</t>
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">timestamptz</t>
-        </is>
-      </c>
-      <c r="G212" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H212" s="4" t="inlineStr">
@@ -13627,12 +13659,12 @@
       </c>
       <c r="I212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">now()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">view_contacts / manage_contacts / manage_logins</t>
         </is>
       </c>
       <c r="K212" s="4" t="inlineStr">
@@ -13649,32 +13681,32 @@
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ポータル権限機能</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_portal_role_permissions</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者ID</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">contact_id</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G213" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK / FK</t>
+          <t xml:space="preserve">timestamptz</t>
+        </is>
+      </c>
+      <c r="G213" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H213" s="4" t="inlineStr">
@@ -13684,12 +13716,12 @@
       </c>
       <c r="I213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K213" s="4" t="inlineStr">
@@ -13706,32 +13738,32 @@
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">通知種別</t>
+          <t xml:space="preserve">医院ログインID</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">topic</t>
+          <t xml:space="preserve">clinic_user_id</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">uuid</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">PK / FK</t>
         </is>
       </c>
       <c r="H214" s="4" t="inlineStr">
@@ -13746,7 +13778,7 @@
       </c>
       <c r="J214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar / orders / billing / product / system / sales</t>
+          <t xml:space="preserve">clinic_users.id ON DELETE CASCADE</t>
         </is>
       </c>
       <c r="K214" s="4" t="inlineStr">
@@ -13763,22 +13795,22 @@
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">連絡方法</t>
+          <t xml:space="preserve">権限キー</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">channel</t>
+          <t xml:space="preserve">role_key</t>
         </is>
       </c>
       <c r="F215" s="4" t="inlineStr">
@@ -13786,9 +13818,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G215" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK</t>
+      <c r="G215" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
       <c r="H215" s="4" t="inlineStr">
@@ -13803,7 +13835,7 @@
       </c>
       <c r="J215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">email / phone</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K215" s="4" t="inlineStr">
@@ -13820,27 +13852,27 @@
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">有効</t>
+          <t xml:space="preserve">割当操作者</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">enabled</t>
+          <t xml:space="preserve">assigned_by</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolean</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G216" s="4" t="inlineStr">
@@ -13855,7 +13887,7 @@
       </c>
       <c r="I216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
+          <t xml:space="preserve">system</t>
         </is>
       </c>
       <c r="J216" s="4" t="inlineStr">
@@ -13877,12 +13909,12 @@
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
@@ -13934,12 +13966,12 @@
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">医院ログイン権限割当</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences</t>
+          <t xml:space="preserve">clinic_user_role_assignments</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
@@ -13991,22 +14023,22 @@
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベントID</t>
+          <t xml:space="preserve">担当者ID</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">contact_id</t>
         </is>
       </c>
       <c r="F219" s="4" t="inlineStr">
@@ -14016,7 +14048,7 @@
       </c>
       <c r="G219" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK</t>
+          <t xml:space="preserve">PK / FK</t>
         </is>
       </c>
       <c r="H219" s="4" t="inlineStr">
@@ -14026,12 +14058,12 @@
       </c>
       <c r="I219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">gen_random_uuid()</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
         </is>
       </c>
       <c r="K219" s="4" t="inlineStr">
@@ -14048,32 +14080,32 @@
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者ID</t>
+          <t xml:space="preserve">通知種別</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">contact_id</t>
+          <t xml:space="preserve">topic</t>
         </is>
       </c>
       <c r="F220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uuid</t>
-        </is>
-      </c>
-      <c r="G220" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G220" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr">
@@ -14088,7 +14120,7 @@
       </c>
       <c r="J220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
+          <t xml:space="preserve">webinar / orders / billing / product / system / sales</t>
         </is>
       </c>
       <c r="K220" s="4" t="inlineStr">
@@ -14105,22 +14137,22 @@
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">イベント種別</t>
+          <t xml:space="preserve">連絡方法</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">event_type</t>
+          <t xml:space="preserve">channel</t>
         </is>
       </c>
       <c r="F221" s="4" t="inlineStr">
@@ -14128,9 +14160,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="G221" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="G221" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
         </is>
       </c>
       <c r="H221" s="4" t="inlineStr">
@@ -14145,7 +14177,7 @@
       </c>
       <c r="J221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">email / phone</t>
         </is>
       </c>
       <c r="K221" s="4" t="inlineStr">
@@ -14162,27 +14194,27 @@
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者種別</t>
+          <t xml:space="preserve">有効</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_type</t>
+          <t xml:space="preserve">enabled</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">boolean</t>
         </is>
       </c>
       <c r="G222" s="4" t="inlineStr">
@@ -14197,7 +14229,7 @@
       </c>
       <c r="I222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">true</t>
         </is>
       </c>
       <c r="J222" s="4" t="inlineStr">
@@ -14219,27 +14251,27 @@
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">操作者識別子</t>
+          <t xml:space="preserve">作成日時</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor_identifier</t>
+          <t xml:space="preserve">created_at</t>
         </is>
       </c>
       <c r="F223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G223" s="4" t="inlineStr">
@@ -14254,7 +14286,7 @@
       </c>
       <c r="I223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J223" s="4" t="inlineStr">
@@ -14276,27 +14308,27 @@
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者操作履歴</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_events</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">追加情報</t>
+          <t xml:space="preserve">更新日時</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">metadata</t>
+          <t xml:space="preserve">updated_at</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">jsonb</t>
+          <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
       <c r="G224" s="4" t="inlineStr">
@@ -14311,7 +14343,7 @@
       </c>
       <c r="I224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">{}</t>
+          <t xml:space="preserve">now()</t>
         </is>
       </c>
       <c r="J224" s="4" t="inlineStr">
@@ -14343,40 +14375,382 @@
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">イベントID</t>
+        </is>
+      </c>
+      <c r="E225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="F225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G225" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK</t>
+        </is>
+      </c>
+      <c r="H225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="J225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="30" customHeight="1">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者ID</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">contact_id</t>
+        </is>
+      </c>
+      <c r="F226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uuid</t>
+        </is>
+      </c>
+      <c r="G226" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+      <c r="H226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id ON DELETE RESTRICT</t>
+        </is>
+      </c>
+      <c r="K226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="30" customHeight="1">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">イベント種別</t>
+        </is>
+      </c>
+      <c r="E227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">event_type</t>
+        </is>
+      </c>
+      <c r="F227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K227" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="30" customHeight="1">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者種別</t>
+        </is>
+      </c>
+      <c r="E228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_type</t>
+        </is>
+      </c>
+      <c r="F228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K228" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="30" customHeight="1">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">操作者識別子</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actor_identifier</t>
+        </is>
+      </c>
+      <c r="F229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="30" customHeight="1">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">追加情報</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metadata</t>
+        </is>
+      </c>
+      <c r="F230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jsonb</t>
+        </is>
+      </c>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="I230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="J230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="30" customHeight="1">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者操作履歴</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contact_events</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">発生日時</t>
         </is>
       </c>
-      <c r="E225" s="4" t="inlineStr">
+      <c r="E231" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">created_at</t>
         </is>
       </c>
-      <c r="F225" s="4" t="inlineStr">
+      <c r="F231" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">timestamptz</t>
         </is>
       </c>
-      <c r="G225" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H225" s="4" t="inlineStr">
+      <c r="G231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H231" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">NO</t>
         </is>
       </c>
-      <c r="I225" s="4" t="inlineStr">
+      <c r="I231" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">now()</t>
         </is>
       </c>
-      <c r="J225" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K225" s="4" t="inlineStr">
+      <c r="J231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K231" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -14387,7 +14761,7 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <autoFilter ref="A4:K225"/>
+  <autoFilter ref="A4:K231"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
 </worksheet>
@@ -19112,7 +19486,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -19733,17 +20107,17 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_id WHERE deleted_at IS NULL</t>
+          <t xml:space="preserve">clinic_user_id</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARTIAL UNIQUE</t>
+          <t xml:space="preserve">UNIQUE</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1ログインと複数担当者の誤関連防止。</t>
+          <t xml:space="preserve">1担当者と1認証アカウントを必須の一対一にする。</t>
         </is>
       </c>
     </row>
@@ -19775,7 +20149,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ログインIDの重複防止。</t>
+          <t xml:space="preserve">担当者ID兼ログインIDの重複防止。</t>
         </is>
       </c>
     </row>
@@ -20901,12 +21275,12 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id</t>
+          <t xml:space="preserve">clinic_contact_roles.role_key</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -20916,12 +21290,12 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.clinic_user_id</t>
+          <t xml:space="preserve">clinic_contacts.role_key</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -20931,19 +21305,19 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・SET NULL</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">医院認証アカウント</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">clinic_users.(id, customer_code)</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -20953,34 +21327,34 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.customer_code</t>
+          <t xml:space="preserve">clinic_contacts.(clinic_user_id, customer_code)</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">UK・複合FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -20995,29 +21369,29 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
+          <t xml:space="preserve">clinic_users.customer_code</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限機能</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -21027,34 +21401,34 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
+          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限割当</t>
+          <t xml:space="preserve">権限機能</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key</t>
+          <t xml:space="preserve">clinic_users.id</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -21064,12 +21438,12 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
+          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -21079,19 +21453,19 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.id</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -21106,17 +21480,17 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
+          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">権限割当</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
@@ -21143,98 +21517,98 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">clinic_contact_events.contact_id</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">将来リレーション案</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親DB日本語名</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親KEY</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">親多重度</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子多重度</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子FK</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">子DB日本語名</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">削除・備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.id</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">order_transaction_projections.order_id</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">決済返金投影</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
@@ -21261,12 +21635,12 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.order_id</t>
+          <t xml:space="preserve">order_transaction_projections.order_id</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">決済返金投影</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -21278,32 +21652,32 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">患者注文</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.id</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillments.order_id</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">受取配送</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_fulfillments.id</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -21315,12 +21689,12 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文明細</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.id</t>
+          <t xml:space="preserve">patient_fulfillments.id</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -21335,7 +21709,7 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
+          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -21352,12 +21726,12 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">注文明細</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
+          <t xml:space="preserve">patient_order_items.id</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -21372,12 +21746,12 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.commerce_account_id</t>
+          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -21409,12 +21783,12 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
+          <t xml:space="preserve">patient_orders.commerce_account_id</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部受信イベント</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -21446,12 +21820,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
+          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部送信キュー</t>
+          <t xml:space="preserve">外部受信イベント</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -21463,12 +21837,12 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">commerce_accounts.id</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -21483,12 +21857,12 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">外部送信キュー</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -21500,32 +21874,32 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">患者</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patients.id</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">患者定期購入</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscriptions.id</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">定期購入明細</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -21547,25 +21921,62 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">定期購入明細</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者定期購入</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_subscriptions.id</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">0..1</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_orders.subscription_id</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="F77" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">患者注文</t>
         </is>
       </c>
-      <c r="G76" s="4" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
@@ -21576,7 +21987,7 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A66:H66"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
@@ -21585,7 +21996,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q103"/>
+  <dimension ref="A1:Q104"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -23568,12 +23979,12 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ログイン</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id</t>
+          <t xml:space="preserve">clinic_contact_roles.role_key</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -23583,12 +23994,12 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.clinic_user_id</t>
+          <t xml:space="preserve">clinic_contacts.role_key</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -23598,19 +24009,19 @@
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・SET NULL</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">医院認証アカウント</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">clinic_users.(id, customer_code)</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -23620,34 +24031,34 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.customer_code</t>
+          <t xml:space="preserve">clinic_contacts.(clinic_user_id, customer_code)</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">UK・複合FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -23662,29 +24073,29 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
+          <t xml:space="preserve">clinic_users.customer_code</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限機能</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -23694,34 +24105,34 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
+          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限割当</t>
+          <t xml:space="preserve">権限機能</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key</t>
+          <t xml:space="preserve">clinic_users.id</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -23731,12 +24142,12 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
+          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
         </is>
       </c>
       <c r="F101" s="4" t="inlineStr">
@@ -23746,19 +24157,19 @@
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.id</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -23773,17 +24184,17 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
+          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者通知設定</t>
+          <t xml:space="preserve">権限割当</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
@@ -23810,15 +24221,52 @@
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">担当者通知設定</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院業務連絡担当者</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_contacts.id</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">clinic_contact_events.contact_id</t>
         </is>
       </c>
-      <c r="F103" s="4" t="inlineStr">
+      <c r="F104" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
-      <c r="G103" s="4" t="inlineStr">
+      <c r="G104" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK・RESTRICT</t>
         </is>

</xml_diff>

<commit_message>
feat: allow duplicate clinic contact emails
</commit_message>
<xml_diff>
--- a/project_clinic_order_management_db_definition.xlsx
+++ b/project_clinic_order_management_db_definition.xlsx
@@ -19486,7 +19486,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -20065,7 +20065,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK11</t>
+          <t xml:space="preserve">UK12</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -20075,17 +20075,17 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">customer_code, lower(email) WHERE deleted_at IS NULL</t>
+          <t xml:space="preserve">clinic_user_id</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARTIAL UNIQUE</t>
+          <t xml:space="preserve">UNIQUE</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院内の担当者メール重複防止。</t>
+          <t xml:space="preserve">1担当者と1認証アカウントを必須の一対一にする。</t>
         </is>
       </c>
     </row>
@@ -20097,17 +20097,17 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK12</t>
+          <t xml:space="preserve">UK13</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts</t>
+          <t xml:space="preserve">clinic_users</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_id</t>
+          <t xml:space="preserve">login_id</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -20117,29 +20117,29 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1担当者と1認証アカウントを必須の一対一にする。</t>
+          <t xml:space="preserve">担当者ID兼ログインIDの重複防止。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">現行</t>
+          <t xml:space="preserve">将来案</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK13</t>
+          <t xml:space="preserve">UK1</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">commerce_accounts</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">login_id</t>
+          <t xml:space="preserve">provider, external_account_id</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -20149,39 +20149,39 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">担当者ID兼ログインIDの重複防止。</t>
+          <t xml:space="preserve">外部接続先の重複防止。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">現行</t>
+          <t xml:space="preserve">将来案</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK14</t>
+          <t xml:space="preserve">UK2</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users</t>
+          <t xml:space="preserve">patient_fulfillment_items</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">email WHERE email IS NOT NULL</t>
+          <t xml:space="preserve">fulfillment_id, order_item_id</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARTIAL UNIQUE</t>
+          <t xml:space="preserve">UNIQUE</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">パスワード再設定先の重複防止。</t>
+          <t xml:space="preserve">同一配送への明細重複防止。</t>
         </is>
       </c>
     </row>
@@ -20193,17 +20193,17 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK1</t>
+          <t xml:space="preserve">UK3</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts</t>
+          <t xml:space="preserve">patient_subscriptions</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">provider, external_account_id</t>
+          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -20213,7 +20213,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部接続先の重複防止。</t>
+          <t xml:space="preserve">外部契約の重複防止。</t>
         </is>
       </c>
     </row>
@@ -20225,17 +20225,17 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK2</t>
+          <t xml:space="preserve">UK4</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items</t>
+          <t xml:space="preserve">commerce_webhook_events</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">fulfillment_id, order_item_id</t>
+          <t xml:space="preserve">commerce_account_id, external_event_id</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -20245,7 +20245,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一配送への明細重複防止。</t>
+          <t xml:space="preserve">Webhook重複配信の無害化。</t>
         </is>
       </c>
     </row>
@@ -20257,17 +20257,17 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK3</t>
+          <t xml:space="preserve">UK5</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions</t>
+          <t xml:space="preserve">patient_orders</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_subscription_id</t>
+          <t xml:space="preserve">commerce_account_id, external_order_id</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -20277,7 +20277,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部契約の重複防止。</t>
+          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
         </is>
       </c>
     </row>
@@ -20289,17 +20289,17 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK4</t>
+          <t xml:space="preserve">UK6</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events</t>
+          <t xml:space="preserve">commerce_outbox</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_account_id, external_event_id</t>
+          <t xml:space="preserve">idempotency_key</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -20309,127 +20309,137 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook重複配信の無害化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将来案</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK5</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_account_id, external_order_id</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UNIQUE</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">複数ストアを考慮した外部注文の一意性。</t>
+          <t xml:space="preserve">外部送信コマンドの二重実行防止。</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将来案</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UK6</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commerce_outbox</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">idempotency_key</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UNIQUE</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部送信コマンドの二重実行防止。</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">現行リレーション</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親DB日本語名</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親KEY</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親多重度</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子多重度</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子FK</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子DB日本語名</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">削除・備考</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">現行リレーション</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0..1</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_terms.customer_code</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院契約情報</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親DB日本語名</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親KEY</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親多重度</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子多重度</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子FK</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子DB日本語名</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">削除・備考</t>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinics.customer_code</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinic_product_settings.customer_code</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院商品設定</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">商品</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">products.id</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -20439,17 +20449,17 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_terms.customer_code</t>
+          <t xml:space="preserve">clinic_product_settings.product_id</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院契約情報</t>
+          <t xml:space="preserve">医院商品設定</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -20481,29 +20491,29 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_product_settings.customer_code</t>
+          <t xml:space="preserve">patient_orders.customer_code</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院商品設定</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">商品</t>
+          <t xml:space="preserve">患者</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">products.id</t>
+          <t xml:space="preserve">patients.id</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -20518,29 +20528,29 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_product_settings.product_id</t>
+          <t xml:space="preserve">patient_orders.patient_id</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院商品設定</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・現状CASCADE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -20555,29 +20565,29 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.customer_code</t>
+          <t xml:space="preserve">patient_order_items.order_id</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -20592,29 +20602,29 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.patient_id</t>
+          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・現状CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">患者</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">patients.id</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -20629,29 +20639,29 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.order_id</t>
+          <t xml:space="preserve">delivery_destinations.patient_id</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">delivery_destinations.id</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -20666,12 +20676,12 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.clinic_customer_code</t>
+          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -20683,12 +20693,12 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -20698,34 +20708,34 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.patient_id</t>
+          <t xml:space="preserve">order_delivery_destinations.order_id</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">注文配送先</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.id</t>
+          <t xml:space="preserve">patient_orders.id</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -20740,66 +20750,66 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations.delivery_destination_id</t>
+          <t xml:space="preserve">patient_order_events.order_id</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">注文操作履歴</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">商品</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">products.id</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_delivery_destinations.order_id</t>
+          <t xml:space="preserve">patient_order_items.product_id</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文配送先</t>
+          <t xml:space="preserve">患者注文明細</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・SET NULL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -20814,34 +20824,34 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_events.order_id</t>
+          <t xml:space="preserve">patient_subscription_requests.customer_code</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文操作履歴</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">商品</t>
+          <t xml:space="preserve">患者</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">products.id</t>
+          <t xml:space="preserve">patients.id</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -20851,29 +20861,29 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.product_id</t>
+          <t xml:space="preserve">patient_subscription_requests.patient_id</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文明細</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・SET NULL</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">patient_subscription_requests.id</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -20888,29 +20898,29 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.customer_code</t>
+          <t xml:space="preserve">patient_subscription_request_items.request_id</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">定期購入申込明細</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">定期購入申込</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_subscription_requests.id</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -20920,22 +20930,22 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.patient_id</t>
+          <t xml:space="preserve">patient_subscription_request_destinations.request_id</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">定期購入申込配送先</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -20962,12 +20972,12 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_items.request_id</t>
+          <t xml:space="preserve">patient_subscription_request_events.request_id</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込明細</t>
+          <t xml:space="preserve">定期購入申込履歴</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -20979,12 +20989,12 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">送り先マスタ</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.id</t>
+          <t xml:space="preserve">delivery_destinations.id</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -20994,12 +21004,12 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_destinations.request_id</t>
+          <t xml:space="preserve">patient_subscription_request_destinations.delivery_destination_id</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -21009,19 +21019,19 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込</t>
+          <t xml:space="preserve">ウェビナー</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_requests.id</t>
+          <t xml:space="preserve">webinars.id</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -21036,12 +21046,12 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_events.request_id</t>
+          <t xml:space="preserve">webinar_sessions.webinar_id</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込履歴</t>
+          <t xml:space="preserve">ウェビナー開催枠</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -21053,12 +21063,12 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">送り先マスタ</t>
+          <t xml:space="preserve">ウェビナー</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery_destinations.id</t>
+          <t xml:space="preserve">webinars.id</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -21073,29 +21083,29 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscription_request_destinations.delivery_destination_id</t>
+          <t xml:space="preserve">webinar_target_clinics.webinar_id</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">定期購入申込配送先</t>
+          <t xml:space="preserve">ウェビナー対象医院</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinars.id</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -21110,17 +21120,17 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_sessions.webinar_id</t>
+          <t xml:space="preserve">webinar_target_clinics.customer_code</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー開催枠</t>
+          <t xml:space="preserve">ウェビナー対象医院</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
@@ -21147,17 +21157,17 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_target_clinics.webinar_id</t>
+          <t xml:space="preserve">webinar_events.webinar_id</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー対象医院</t>
+          <t xml:space="preserve">ウェビナー操作履歴</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -21184,29 +21194,29 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_target_clinics.customer_code</t>
+          <t xml:space="preserve">clinic_contacts.customer_code</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー対象医院</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー</t>
+          <t xml:space="preserve">医院担当者役職</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinars.id</t>
+          <t xml:space="preserve">clinic_contact_roles.role_key</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -21221,29 +21231,29 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">webinar_events.webinar_id</t>
+          <t xml:space="preserve">clinic_contacts.role_key</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ウェビナー操作履歴</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">医院認証アカウント</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">clinic_users.(id, customer_code)</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -21253,12 +21263,12 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.customer_code</t>
+          <t xml:space="preserve">clinic_contacts.(clinic_user_id, customer_code)</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -21268,19 +21278,19 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">UK・複合FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院担当者役職</t>
+          <t xml:space="preserve">医院</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contact_roles.role_key</t>
+          <t xml:space="preserve">clinics.customer_code</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -21295,29 +21305,29 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.role_key</t>
+          <t xml:space="preserve">clinic_users.customer_code</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
+          <t xml:space="preserve">FK・CASCADE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院認証アカウント</t>
+          <t xml:space="preserve">医院ポータル権限</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.(id, customer_code)</t>
+          <t xml:space="preserve">clinic_portal_roles.role_key</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -21327,34 +21337,34 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_contacts.(clinic_user_id, customer_code)</t>
+          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
+          <t xml:space="preserve">権限機能</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UK・複合FK・RESTRICT</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院</t>
+          <t xml:space="preserve">医院ポータルログイン</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinics.customer_code</t>
+          <t xml:space="preserve">clinic_users.id</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -21364,22 +21374,22 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.customer_code</t>
+          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">権限割当</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・CASCADE</t>
         </is>
       </c>
     </row>
@@ -21406,29 +21416,29 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_role_permissions.role_key</t>
+          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限機能</t>
+          <t xml:space="preserve">権限割当</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
+          <t xml:space="preserve">FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータルログイン</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_users.id</t>
+          <t xml:space="preserve">clinic_contacts.id</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -21438,34 +21448,34 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0..1</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.clinic_user_id</t>
+          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限割当</t>
+          <t xml:space="preserve">担当者通知設定</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PK・FK・CASCADE</t>
+          <t xml:space="preserve">PK・FK・RESTRICT</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">医院ポータル権限</t>
+          <t xml:space="preserve">医院業務連絡担当者</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_portal_roles.role_key</t>
+          <t xml:space="preserve">clinic_contacts.id</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -21480,12 +21490,12 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">clinic_user_role_assignments.role_key</t>
+          <t xml:space="preserve">clinic_contact_events.contact_id</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">権限割当</t>
+          <t xml:space="preserve">担当者操作履歴</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -21494,133 +21504,133 @@
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_contacts.id</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将来リレーション案</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親DB日本語名</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親KEY</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">親多重度</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子多重度</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子FK</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">子DB日本語名</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">削除・備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者注文</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.id</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_contact_notification_preferences.contact_id</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">担当者通知設定</t>
-        </is>
-      </c>
-      <c r="G63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PK・FK・RESTRICT</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">医院業務連絡担当者</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_contacts.id</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order_transaction_projections.order_id</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">決済返金投影</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">患者注文</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_orders.id</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">clinic_contact_events.contact_id</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">担当者操作履歴</t>
-        </is>
-      </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK・RESTRICT</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将来リレーション案</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親DB日本語名</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親KEY</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">親多重度</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子多重度</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子FK</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">子DB日本語名</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">削除・備考</t>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">patient_fulfillments.order_id</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受取配送</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FK</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">受取配送</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">patient_fulfillments.id</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -21635,12 +21645,12 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">order_transaction_projections.order_id</t>
+          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">決済返金投影</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -21652,12 +21662,12 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">注文明細</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.id</t>
+          <t xml:space="preserve">patient_order_items.id</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -21672,12 +21682,12 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.order_id</t>
+          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">受取配送明細</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -21689,12 +21699,12 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillments.id</t>
+          <t xml:space="preserve">commerce_accounts.id</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -21709,12 +21719,12 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.fulfillment_id</t>
+          <t xml:space="preserve">patient_orders.commerce_account_id</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -21726,12 +21736,12 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">注文明細</t>
+          <t xml:space="preserve">外部コマース接続</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_order_items.id</t>
+          <t xml:space="preserve">commerce_accounts.id</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -21746,12 +21756,12 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_fulfillment_items.order_item_id</t>
+          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">受取配送明細</t>
+          <t xml:space="preserve">外部受信イベント</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -21783,12 +21793,12 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_orders.commerce_account_id</t>
+          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者注文</t>
+          <t xml:space="preserve">外部送信キュー</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -21800,12 +21810,12 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">患者</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
+          <t xml:space="preserve">patients.id</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -21820,12 +21830,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_webhook_events.commerce_account_id</t>
+          <t xml:space="preserve">patient_subscriptions.patient_id</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部受信イベント</t>
+          <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -21837,12 +21847,12 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部コマース接続</t>
+          <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_accounts.id</t>
+          <t xml:space="preserve">patient_subscriptions.id</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -21857,12 +21867,12 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">commerce_outbox.commerce_account_id</t>
+          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">外部送信キュー</t>
+          <t xml:space="preserve">定期購入明細</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -21874,17 +21884,17 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者</t>
+          <t xml:space="preserve">患者定期購入</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patients.id</t>
+          <t xml:space="preserve">patient_subscriptions.id</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0..1</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -21894,89 +21904,15 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient_subscriptions.patient_id</t>
+          <t xml:space="preserve">patient_orders.subscription_id</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">患者定期購入</t>
+          <t xml:space="preserve">患者注文</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者定期購入</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscriptions.id</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscription_items.subscription_id</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">定期購入明細</t>
-        </is>
-      </c>
-      <c r="G76" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者定期購入</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_subscriptions.id</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0..1</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">patient_orders.subscription_id</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">患者注文</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FK</t>
         </is>
@@ -21986,8 +21922,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A64:H64"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>

</xml_diff>